<commit_message>
docs: prepare OTEL customer telemetry branch
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
Copilot-Session-Id: 76441afe-520c-42ec-8343-5c5bd3393dbe
</commit_message>
<xml_diff>
--- a/docs/lineage/model-storage-checker-lineage-run-2.xlsx
+++ b/docs/lineage/model-storage-checker-lineage-run-2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="211">
   <si>
     <t>Model Storage Checker — Copilot Lineage Run 2</t>
     <phoneticPr fontId="1"/>
@@ -794,6 +794,74 @@
   </si>
   <si>
     <t>No release created; placeholder remains null</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>53 / 53 passed</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>See telemetry/run-2/artifact-integrity.json</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>docs/lineage/index.html on the OTEL branch</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Customer branch</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OTEL</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Merged main SHA</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>94c7a17e32e0cbc699ff1cd031b099df6d379cc7</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>All five PRs are merged into main through native stack #11 and verified against the approved titles, bases, heads, and SHAs.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>MERGED</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>53 / 53 tests</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>0 matches; see sanitization-validation.json</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>All integrity records verified; see artifact-integrity.json</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>index.html, data.json, workbook, and vendored Cytoscape returned HTTP 200</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Render, primary path, and expansion checks passed</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Pull request landing</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PRs #6–#10 merged via native stack #11; exact approved head SHAs</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Merged at 94c7a17e32e0cbc699ff1cd031b099df6d379cc7</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1267,7 +1335,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="6" width="8.38" customWidth="1"/>
@@ -1410,7 +1478,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s" s="6">
-        <v>23</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1418,7 +1486,7 @@
         <v>24</v>
       </c>
       <c r="B19" t="s" s="6">
-        <v>25</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -1434,7 +1502,7 @@
         <v>28</v>
       </c>
       <c r="B21" t="s" s="6">
-        <v>29</v>
+        <v>196</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -1443,6 +1511,22 @@
       </c>
       <c r="B22" t="s" s="6">
         <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>197</v>
+      </c>
+      <c r="B23" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2202,7 +2286,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s" s="3">
-        <v>126</v>
+        <v>201</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2255,7 +2339,7 @@
         <v>57</v>
       </c>
       <c r="F4" t="s" s="6">
-        <v>135</v>
+        <v>202</v>
       </c>
       <c r="G4" t="b" s="6">
         <v>0</v>
@@ -2281,7 +2365,7 @@
         <v>65</v>
       </c>
       <c r="F5" t="s" s="6">
-        <v>135</v>
+        <v>202</v>
       </c>
       <c r="G5" t="b" s="6">
         <v>0</v>
@@ -2307,7 +2391,7 @@
         <v>71</v>
       </c>
       <c r="F6" t="s" s="6">
-        <v>135</v>
+        <v>202</v>
       </c>
       <c r="G6" t="b" s="6">
         <v>0</v>
@@ -2333,7 +2417,7 @@
         <v>77</v>
       </c>
       <c r="F7" t="s" s="6">
-        <v>135</v>
+        <v>202</v>
       </c>
       <c r="G7" t="b" s="6">
         <v>0</v>
@@ -2359,7 +2443,7 @@
         <v>83</v>
       </c>
       <c r="F8" t="s" s="6">
-        <v>135</v>
+        <v>202</v>
       </c>
       <c r="G8" t="b" s="6">
         <v>0</v>
@@ -2387,126 +2471,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s" s="25">
+      <c r="A1" t="s" s="8">
         <v>140</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s" s="26">
+      <c r="A2" t="s" s="3">
         <v>141</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s" s="27">
+      <c r="A3" t="s" s="4">
         <v>142</v>
       </c>
-      <c r="B3" t="s" s="27">
+      <c r="B3" t="s" s="4">
         <v>143</v>
       </c>
-      <c r="C3" t="s" s="27">
+      <c r="C3" t="s" s="4">
         <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" t="s" s="28">
+      <c r="A4" t="s" s="6">
         <v>145</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="12">
         <v>163</v>
       </c>
-      <c r="C4" t="s" s="28">
+      <c r="C4" t="s" s="6">
         <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" t="s" s="28">
+      <c r="A5" t="s" s="6">
         <v>147</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="12">
         <v>163</v>
       </c>
-      <c r="C5" t="s" s="28">
+      <c r="C5" t="s" s="6">
         <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" t="s" s="28">
+      <c r="A6" t="s" s="6">
         <v>149</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="12">
         <v>240</v>
       </c>
-      <c r="C6" t="s" s="28">
+      <c r="C6" t="s" s="6">
         <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" t="s" s="28">
+      <c r="A7" t="s" s="6">
         <v>151</v>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="12">
         <v>30</v>
       </c>
-      <c r="C7" t="s" s="28">
+      <c r="C7" t="s" s="6">
         <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" t="s" s="28">
+      <c r="A8" t="s" s="6">
         <v>153</v>
       </c>
-      <c r="B8" s="29">
+      <c r="B8" s="12">
         <v>33</v>
       </c>
-      <c r="C8" t="s" s="28">
+      <c r="C8" t="s" s="6">
         <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" t="s" s="28">
+      <c r="A9" t="s" s="6">
         <v>155</v>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="12">
         <v>154</v>
       </c>
-      <c r="C9" t="s" s="28">
+      <c r="C9" t="s" s="6">
         <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" t="s" s="28">
+      <c r="A10" t="s" s="6">
         <v>157</v>
       </c>
-      <c r="B10" s="29">
+      <c r="B10" s="12">
         <v>86</v>
       </c>
-      <c r="C10" t="s" s="28">
+      <c r="C10" t="s" s="6">
         <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" t="s" s="28">
+      <c r="A11" t="s" s="6">
         <v>159</v>
       </c>
-      <c r="B11" s="29">
+      <c r="B11" s="12">
         <v>43</v>
       </c>
-      <c r="C11" t="s" s="28">
+      <c r="C11" t="s" s="6">
         <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" t="s" s="28">
+      <c r="A12" t="s" s="6">
         <v>161</v>
       </c>
-      <c r="B12" s="29">
+      <c r="B12" s="12">
         <v>7</v>
       </c>
-      <c r="C12" t="s" s="28">
+      <c r="C12" t="s" s="6">
         <v>162</v>
       </c>
     </row>
@@ -2540,159 +2624,159 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s" s="25">
+      <c r="A1" t="s" s="8">
         <v>165</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s" s="26">
+      <c r="A2" t="s" s="3">
         <v>166</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s" s="27">
+      <c r="A3" t="s" s="4">
         <v>167</v>
       </c>
-      <c r="B3" t="s" s="27">
+      <c r="B3" t="s" s="4">
         <v>168</v>
       </c>
-      <c r="C3" t="s" s="27">
+      <c r="C3" t="s" s="4">
         <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" t="s" s="28">
+      <c r="A4" t="s" s="6">
         <v>20</v>
       </c>
       <c r="B4" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C4" t="s" s="28">
+      <c r="C4" t="s" s="6">
         <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" t="s" s="28">
+      <c r="A5" t="s" s="6">
         <v>22</v>
       </c>
       <c r="B5" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C5" t="s" s="28">
-        <v>172</v>
+      <c r="C5" t="s" s="6">
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" t="s" s="28">
+      <c r="A6" t="s" s="6">
         <v>173</v>
       </c>
       <c r="B6" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C6" t="s" s="28">
+      <c r="C6" t="s" s="6">
         <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" t="s" s="28">
+      <c r="A7" t="s" s="6">
         <v>175</v>
       </c>
       <c r="B7" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C7" t="s" s="28">
+      <c r="C7" t="s" s="6">
         <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" t="s" s="28">
+      <c r="A8" t="s" s="6">
         <v>177</v>
       </c>
       <c r="B8" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C8" t="s" s="28">
-        <v>178</v>
+      <c r="C8" t="s" s="6">
+        <v>204</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" t="s" s="28">
+      <c r="A9" t="s" s="6">
         <v>179</v>
       </c>
       <c r="B9" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C9" t="s" s="28">
-        <v>180</v>
+      <c r="C9" t="s" s="6">
+        <v>205</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" t="s" s="28">
+      <c r="A10" t="s" s="6">
         <v>181</v>
       </c>
       <c r="B10" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C10" t="s" s="28">
-        <v>182</v>
+      <c r="C10" t="s" s="6">
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" t="s" s="28">
+      <c r="A11" t="s" s="6">
         <v>183</v>
       </c>
       <c r="B11" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C11" t="s" s="28">
-        <v>184</v>
+      <c r="C11" t="s" s="6">
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" t="s" s="28">
-        <v>185</v>
+      <c r="A12" t="s" s="6">
+        <v>208</v>
       </c>
       <c r="B12" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C12" t="s" s="28">
-        <v>186</v>
+      <c r="C12" t="s" s="6">
+        <v>209</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" t="s" s="28">
+      <c r="A13" t="s" s="6">
         <v>187</v>
       </c>
       <c r="B13" t="s" s="32">
         <v>170</v>
       </c>
-      <c r="C13" t="s" s="28">
-        <v>188</v>
+      <c r="C13" t="s" s="6">
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" t="s" s="28">
+      <c r="A14" t="s" s="6">
         <v>189</v>
       </c>
       <c r="B14" t="s" s="33">
         <v>190</v>
       </c>
-      <c r="C14" t="s" s="28">
+      <c r="C14" t="s" s="6">
         <v>191</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" t="s" s="28">
+      <c r="A15" t="s" s="6">
         <v>30</v>
       </c>
       <c r="B15" t="s" s="33">
         <v>192</v>
       </c>
-      <c r="C15" t="s" s="28">
+      <c r="C15" t="s" s="6">
         <v>193</v>
       </c>
     </row>

</xml_diff>